<commit_message>
Setting up workflow spreadsheet for public users
</commit_message>
<xml_diff>
--- a/W3_LSPC_Watershed/inputs/LSPC_Workflow_Control_File.xlsx
+++ b/W3_LSPC_Watershed/inputs/LSPC_Workflow_Control_File.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aprashar\Documents\Github\DWRAT_DataScraping\W3_LSPC_Watershed\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96FEC62B-509D-446D-B204-95F475B8392F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBC14620-5D13-4F93-92A0-3159A37A6A1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-24525" yWindow="-16395" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="22">
   <si>
     <t>CATEGORY</t>
   </si>
@@ -68,10 +68,40 @@
     <t>An optional field with a text file that contains login credentials for the NASA Earthdata website (required for gathering NLDAS data); on the first line, there should be a username, and on the second line, there should be a password</t>
   </si>
   <si>
-    <t>HISTORIC_WEATHER_DATA_LOCATION</t>
-  </si>
-  <si>
-    <t>The path to a folder that contains historic weather data for each watershed (every .air and .pre file should have a counterpart here); for the model run, these files will be copied and merged with (1) the downloaded meteorological data and (2) predictions for the remainder of the water year</t>
+    <t>HISTORIC_SHARED_WEATHER_DATA_LOCATION</t>
+  </si>
+  <si>
+    <t>The path to a folder that contains raw historic weather data (with separate folders for each source); for the model run, these files will be copied and stored in the "data\shared\raw" folder</t>
+  </si>
+  <si>
+    <t>PRIOR_MANUAL_REVIEW_SHEETS_LOCATION</t>
+  </si>
+  <si>
+    <t>An optional field containing the path to a folder that contains completed manual review sheets (with separate folders for each watershed); for the model run, these spreadsheets' manual review edits will be integrated into the newly generated sheets</t>
+  </si>
+  <si>
+    <t>DWRAT</t>
+  </si>
+  <si>
+    <t>SUBWATERSHED_TYPE</t>
+  </si>
+  <si>
+    <t>AUTO</t>
+  </si>
+  <si>
+    <t>ADDITIONAL_ARCHIVE_LOCATION</t>
+  </si>
+  <si>
+    <t>This is an optional field that identifies another folder where archived files in the "HYDROLOGY_OUTPUT_LOCATION" directory will be copied to</t>
+  </si>
+  <si>
+    <t>LONG-RUNNING_METADATA_FILE_LOCATION</t>
+  </si>
+  <si>
+    <t>This is an optional field that requires a folder path; "LSPC_Workflow_Tracker.csv" will either be generated or updated by the scripts here, and the file will contain metadata from multiple workflow runs (after each run, this CSV file will be updated automatically)</t>
+  </si>
+  <si>
+    <t>Either "CATCHMENT", "HUC12", or "AUTO"; this affects how LSPC streamflow data is wrapped up before modeling a watershed in DWRAT</t>
   </si>
 </sst>
 </file>
@@ -116,7 +146,10 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="15">
+  <dxfs count="16">
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -313,23 +346,23 @@
   <tableStyles count="3" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="Table Style 1" pivot="0" count="0" xr9:uid="{CC00AC29-08EF-4179-858D-4AAEFFD3939B}"/>
     <tableStyle name="TableStyleMedium14 2" pivot="0" count="8" xr9:uid="{28372B93-A849-49B7-9168-022A6F278C77}">
-      <tableStyleElement type="wholeTable" dxfId="14"/>
-      <tableStyleElement type="headerRow" dxfId="13"/>
-      <tableStyleElement type="totalRow" dxfId="12"/>
-      <tableStyleElement type="firstColumn" dxfId="11"/>
-      <tableStyleElement type="lastColumn" dxfId="10"/>
-      <tableStyleElement type="firstRowStripe" dxfId="9"/>
-      <tableStyleElement type="secondRowStripe" dxfId="8"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="7"/>
+      <tableStyleElement type="wholeTable" dxfId="15"/>
+      <tableStyleElement type="headerRow" dxfId="14"/>
+      <tableStyleElement type="totalRow" dxfId="13"/>
+      <tableStyleElement type="firstColumn" dxfId="12"/>
+      <tableStyleElement type="lastColumn" dxfId="11"/>
+      <tableStyleElement type="firstRowStripe" dxfId="10"/>
+      <tableStyleElement type="secondRowStripe" dxfId="9"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="8"/>
     </tableStyle>
     <tableStyle name="TableStyleMedium2 2" pivot="0" count="7" xr9:uid="{4E02A1E9-3DFE-4ECF-918F-8EA3F0D27893}">
-      <tableStyleElement type="wholeTable" dxfId="6"/>
-      <tableStyleElement type="headerRow" dxfId="5"/>
-      <tableStyleElement type="totalRow" dxfId="4"/>
-      <tableStyleElement type="firstColumn" dxfId="3"/>
-      <tableStyleElement type="lastColumn" dxfId="2"/>
-      <tableStyleElement type="firstRowStripe" dxfId="1"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="0"/>
+      <tableStyleElement type="wholeTable" dxfId="7"/>
+      <tableStyleElement type="headerRow" dxfId="6"/>
+      <tableStyleElement type="totalRow" dxfId="5"/>
+      <tableStyleElement type="firstColumn" dxfId="4"/>
+      <tableStyleElement type="lastColumn" dxfId="3"/>
+      <tableStyleElement type="firstRowStripe" dxfId="2"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="1"/>
     </tableStyle>
   </tableStyles>
   <colors>
@@ -354,13 +387,13 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4F4A1679-A105-4072-8D1A-C0607922493E}" name="Table1" displayName="Table1" ref="A1:D4" totalsRowShown="0">
-  <autoFilter ref="A1:D4" xr:uid="{4F4A1679-A105-4072-8D1A-C0607922493E}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4F4A1679-A105-4072-8D1A-C0607922493E}" name="Table1" displayName="Table1" ref="A1:D8" totalsRowShown="0">
+  <autoFilter ref="A1:D8" xr:uid="{4F4A1679-A105-4072-8D1A-C0607922493E}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{9E8CE8C3-765B-49E7-BB5F-6D2A3283AA67}" name="CATEGORY"/>
     <tableColumn id="2" xr3:uid="{160E1F17-A808-4C9F-9992-4B3BE2F4C29D}" name="FIELD"/>
     <tableColumn id="3" xr3:uid="{648B45E2-4D53-4F45-9165-9844EB4CE789}" name="VALUE"/>
-    <tableColumn id="4" xr3:uid="{BB620692-69FC-46F4-8A8D-4701148ED4D2}" name="NOTES"/>
+    <tableColumn id="4" xr3:uid="{BB620692-69FC-46F4-8A8D-4701148ED4D2}" name="NOTES" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2 2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -629,10 +662,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="49.109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="61.5546875" customWidth="1"/>
     <col min="4" max="4" width="81.6640625" style="1" customWidth="1"/>
@@ -674,7 +707,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -683,6 +716,53 @@
       </c>
       <c r="D4" s="1" t="s">
         <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>4</v>
+      </c>
+      <c r="B8" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -695,6 +775,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="b2cf8adb-cf25-47fc-8c92-b53f2a7e7f06">
@@ -703,15 +792,6 @@
     <TaxCatchAll xmlns="851dfaa3-aae8-4c03-b90c-7dd4a6526d0d" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -956,20 +1036,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{496CF77A-4899-4D89-A2F1-D8663B7093CD}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{250AEEB6-C5D5-4012-920E-FE9FB722CC2C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="b2cf8adb-cf25-47fc-8c92-b53f2a7e7f06"/>
     <ds:schemaRef ds:uri="851dfaa3-aae8-4c03-b90c-7dd4a6526d0d"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{496CF77A-4899-4D89-A2F1-D8663B7093CD}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>